<commit_message>
excluded some dynamic fits after switching to 150Hz; push before excluding static fits
</commit_message>
<xml_diff>
--- a/results/soae/SOAE Results (rho=1.0, Flattop, BW=150Hz, Mode=phi)/SOAE N_xi Fitted Parameters (rho=1.0, Flattop, BW=150Hz, Mode=phi).xlsx
+++ b/results/soae/SOAE Results (rho=1.0, Flattop, BW=150Hz, Mode=phi)/SOAE N_xi Fitted Parameters (rho=1.0, Flattop, BW=150Hz, Mode=phi).xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M65"/>
+  <dimension ref="A1:M60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -735,34 +735,34 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>3022.723388671875</v>
+        <v>3151.922607421875</v>
       </c>
       <c r="E7" t="n">
-        <v>29.48937221956972</v>
+        <v>21.79625805524918</v>
       </c>
       <c r="F7" t="n">
-        <v>2.544971715602453</v>
+        <v>0.4421872250383178</v>
       </c>
       <c r="G7" t="n">
-        <v>0.009755895074648814</v>
+        <v>0.006915226282499843</v>
       </c>
       <c r="H7" t="n">
-        <v>0.0008419466118335965</v>
+        <v>0.0001402912698418081</v>
       </c>
       <c r="I7" t="n">
-        <v>0.4161331532002926</v>
+        <v>1.167184347414524</v>
       </c>
       <c r="J7" t="n">
-        <v>0.05065969059529257</v>
+        <v>0.02826340340911475</v>
       </c>
       <c r="K7" t="n">
-        <v>0.0001814260831365027</v>
+        <v>7.724709468421015e-05</v>
       </c>
       <c r="L7" t="n">
-        <v>0.03</v>
+        <v>0.01900226757369615</v>
       </c>
       <c r="M7" t="n">
-        <v>90.68170166015625</v>
+        <v>59.8936767578125</v>
       </c>
     </row>
     <row r="8">
@@ -780,34 +780,34 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3151.922607421875</v>
+        <v>3954.034423828125</v>
       </c>
       <c r="E8" t="n">
-        <v>21.79625805524918</v>
+        <v>16.81309925874893</v>
       </c>
       <c r="F8" t="n">
-        <v>0.4421872250383178</v>
+        <v>0.4295716883260556</v>
       </c>
       <c r="G8" t="n">
-        <v>0.006915226282499843</v>
+        <v>0.004252137805737972</v>
       </c>
       <c r="H8" t="n">
-        <v>0.0001402912698418081</v>
+        <v>0.000108641362790707</v>
       </c>
       <c r="I8" t="n">
-        <v>1.167184347414524</v>
+        <v>1.206932070789721</v>
       </c>
       <c r="J8" t="n">
-        <v>0.02826340340911475</v>
+        <v>0.0421395586098858</v>
       </c>
       <c r="K8" t="n">
-        <v>7.724709468421015e-05</v>
+        <v>5.318789996053886e-05</v>
       </c>
       <c r="L8" t="n">
-        <v>0.01900226757369615</v>
+        <v>0.01299319727891157</v>
       </c>
       <c r="M8" t="n">
-        <v>59.8936767578125</v>
+        <v>51.37554931640625</v>
       </c>
     </row>
     <row r="9">
@@ -817,42 +817,42 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ACsb4rearSOAEwf1.mat</t>
+          <t>ACsb24rearSOAEwfA1.mat</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>3954.034423828125</v>
+        <v>2177.545166015625</v>
       </c>
       <c r="E9" t="n">
-        <v>16.81309925874893</v>
+        <v>23.32052373889071</v>
       </c>
       <c r="F9" t="n">
-        <v>0.4295716883260556</v>
+        <v>0.3865925997474151</v>
       </c>
       <c r="G9" t="n">
-        <v>0.004252137805737972</v>
+        <v>0.01070954766075487</v>
       </c>
       <c r="H9" t="n">
-        <v>0.000108641362790707</v>
+        <v>0.0001775359729758373</v>
       </c>
       <c r="I9" t="n">
-        <v>1.206932070789721</v>
+        <v>1.287499509764526</v>
       </c>
       <c r="J9" t="n">
-        <v>0.0421395586098858</v>
+        <v>0.02278950629369229</v>
       </c>
       <c r="K9" t="n">
-        <v>5.318789996053886e-05</v>
+        <v>0.0001382658446843509</v>
       </c>
       <c r="L9" t="n">
-        <v>0.01299319727891157</v>
+        <v>0.02800453514739229</v>
       </c>
       <c r="M9" t="n">
-        <v>51.37554931640625</v>
+        <v>60.98114013671875</v>
       </c>
     </row>
     <row r="10">
@@ -870,34 +870,34 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>1811.480712890625</v>
+        <v>3111.5478515625</v>
       </c>
       <c r="E10" t="n">
-        <v>26.81099058843104</v>
+        <v>19.09397641221516</v>
       </c>
       <c r="F10" t="n">
-        <v>2.304897978952203</v>
+        <v>0.2286437396621853</v>
       </c>
       <c r="G10" t="n">
-        <v>0.01480059400999532</v>
+        <v>0.006136488115593948</v>
       </c>
       <c r="H10" t="n">
-        <v>0.001272383394728073</v>
+        <v>7.348231509516049e-05</v>
       </c>
       <c r="I10" t="n">
-        <v>0.2581939228723503</v>
+        <v>1.299685972179711</v>
       </c>
       <c r="J10" t="n">
-        <v>0.03010417075300892</v>
+        <v>0.01991162713313616</v>
       </c>
       <c r="K10" t="n">
-        <v>9.606701367863948e-05</v>
+        <v>2.581869008378071e-05</v>
       </c>
       <c r="L10" t="n">
-        <v>0.04</v>
+        <v>0.01800453514739229</v>
       </c>
       <c r="M10" t="n">
-        <v>72.459228515625</v>
+        <v>56.02197265625001</v>
       </c>
     </row>
     <row r="11">
@@ -915,34 +915,34 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>2177.545166015625</v>
+        <v>3477.6123046875</v>
       </c>
       <c r="E11" t="n">
-        <v>23.32052373889071</v>
+        <v>20.58259462749211</v>
       </c>
       <c r="F11" t="n">
-        <v>0.3865925997474151</v>
+        <v>0.5614362068544968</v>
       </c>
       <c r="G11" t="n">
-        <v>0.01070954766075487</v>
+        <v>0.0059185995516949</v>
       </c>
       <c r="H11" t="n">
-        <v>0.0001775359729758373</v>
+        <v>0.0001614430125226244</v>
       </c>
       <c r="I11" t="n">
-        <v>1.287499509764526</v>
+        <v>1.35682072682345</v>
       </c>
       <c r="J11" t="n">
-        <v>0.02278950629369229</v>
+        <v>0.05449370381820302</v>
       </c>
       <c r="K11" t="n">
-        <v>0.0001382658446843509</v>
+        <v>9.764902668320788e-05</v>
       </c>
       <c r="L11" t="n">
-        <v>0.02800453514739229</v>
+        <v>0.01900226757369615</v>
       </c>
       <c r="M11" t="n">
-        <v>60.98114013671875</v>
+        <v>66.08251953125</v>
       </c>
     </row>
     <row r="12">
@@ -952,42 +952,42 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ACsb24rearSOAEwfA1.mat</t>
+          <t>ACsb30learSOAEwfA2.mat</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>3111.5478515625</v>
+        <v>1798.0224609375</v>
       </c>
       <c r="E12" t="n">
-        <v>19.09397641221516</v>
+        <v>12.77849738964914</v>
       </c>
       <c r="F12" t="n">
-        <v>0.2286437396621853</v>
+        <v>0.07402634290561354</v>
       </c>
       <c r="G12" t="n">
-        <v>0.006136488115593948</v>
+        <v>0.007106973170394295</v>
       </c>
       <c r="H12" t="n">
-        <v>7.348231509516049e-05</v>
+        <v>4.117097784585836e-05</v>
       </c>
       <c r="I12" t="n">
-        <v>1.299685972179711</v>
+        <v>1.034237874709824</v>
       </c>
       <c r="J12" t="n">
-        <v>0.01991162713313616</v>
+        <v>0.007153963905957183</v>
       </c>
       <c r="K12" t="n">
-        <v>2.581869008378071e-05</v>
+        <v>5.92706793932235e-06</v>
       </c>
       <c r="L12" t="n">
-        <v>0.01800453514739229</v>
+        <v>0.02099773242630385</v>
       </c>
       <c r="M12" t="n">
-        <v>56.02197265625001</v>
+        <v>37.75439453125</v>
       </c>
     </row>
     <row r="13">
@@ -997,42 +997,42 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ACsb24rearSOAEwfA1.mat</t>
+          <t>ACsb30learSOAEwfA2.mat</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3477.6123046875</v>
+        <v>2139.862060546875</v>
       </c>
       <c r="E13" t="n">
-        <v>20.58259462749211</v>
+        <v>7.116088476134931</v>
       </c>
       <c r="F13" t="n">
-        <v>0.5614362068544968</v>
+        <v>0.4580633678528805</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0059185995516949</v>
+        <v>0.003325489342203817</v>
       </c>
       <c r="H13" t="n">
-        <v>0.0001614430125226244</v>
+        <v>0.0002140621006831699</v>
       </c>
       <c r="I13" t="n">
-        <v>1.35682072682345</v>
+        <v>1.190339964047119</v>
       </c>
       <c r="J13" t="n">
-        <v>0.05449370381820302</v>
+        <v>0.1217598077429789</v>
       </c>
       <c r="K13" t="n">
-        <v>9.764902668320788e-05</v>
+        <v>0.0001452979324583457</v>
       </c>
       <c r="L13" t="n">
-        <v>0.01900226757369615</v>
+        <v>0.01099773242630385</v>
       </c>
       <c r="M13" t="n">
-        <v>66.08251953125</v>
+        <v>23.53363037109375</v>
       </c>
     </row>
     <row r="14">
@@ -1050,34 +1050,34 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>1798.0224609375</v>
+        <v>2417.10205078125</v>
       </c>
       <c r="E14" t="n">
-        <v>12.77849738964914</v>
+        <v>8.366156163234193</v>
       </c>
       <c r="F14" t="n">
-        <v>0.07402634290561354</v>
+        <v>0.3265928212955004</v>
       </c>
       <c r="G14" t="n">
-        <v>0.007106973170394295</v>
+        <v>0.003461234150428238</v>
       </c>
       <c r="H14" t="n">
-        <v>4.117097784585836e-05</v>
+        <v>0.0001351175144590771</v>
       </c>
       <c r="I14" t="n">
-        <v>1.034237874709824</v>
+        <v>0.8945628357999161</v>
       </c>
       <c r="J14" t="n">
-        <v>0.007153963905957183</v>
+        <v>0.05453311641316103</v>
       </c>
       <c r="K14" t="n">
-        <v>5.92706793932235e-06</v>
+        <v>3.907749666197293e-05</v>
       </c>
       <c r="L14" t="n">
-        <v>0.02099773242630385</v>
+        <v>0.01199546485260771</v>
       </c>
       <c r="M14" t="n">
-        <v>37.75439453125</v>
+        <v>28.9942626953125</v>
       </c>
     </row>
     <row r="15">
@@ -1095,124 +1095,124 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>2139.862060546875</v>
+        <v>2783.16650390625</v>
       </c>
       <c r="E15" t="n">
-        <v>7.116088476134931</v>
+        <v>7.268278767219267</v>
       </c>
       <c r="F15" t="n">
-        <v>0.4580633678528805</v>
+        <v>0.5142485626019108</v>
       </c>
       <c r="G15" t="n">
-        <v>0.003325489342203817</v>
+        <v>0.0026115141717242</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0002140621006831699</v>
+        <v>0.0001847710375502683</v>
       </c>
       <c r="I15" t="n">
-        <v>1.190339964047119</v>
+        <v>1.141272907820804</v>
       </c>
       <c r="J15" t="n">
-        <v>0.1217598077429789</v>
+        <v>0.1502030086969103</v>
       </c>
       <c r="K15" t="n">
-        <v>0.0001452979324583457</v>
+        <v>5.226451848124019e-05</v>
       </c>
       <c r="L15" t="n">
-        <v>0.01099773242630385</v>
+        <v>0.009002267573696146</v>
       </c>
       <c r="M15" t="n">
-        <v>23.53363037109375</v>
+        <v>25.0548095703125</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Anole</t>
+          <t>Tokay</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>ACsb30learSOAEwfA2.mat</t>
+          <t>tokay_GG1rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2417.10205078125</v>
+        <v>1342.7734375</v>
       </c>
       <c r="E16" t="n">
-        <v>8.366156163234193</v>
+        <v>6.131533960577602</v>
       </c>
       <c r="F16" t="n">
-        <v>0.3265928212955004</v>
+        <v>0.4593700147730712</v>
       </c>
       <c r="G16" t="n">
-        <v>0.003461234150428238</v>
+        <v>0.004566320564095612</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0001351175144590771</v>
+        <v>0.0003421053782746363</v>
       </c>
       <c r="I16" t="n">
-        <v>0.8945628357999161</v>
+        <v>0.6492183620177698</v>
       </c>
       <c r="J16" t="n">
-        <v>0.05453311641316103</v>
+        <v>0.06330381715723586</v>
       </c>
       <c r="K16" t="n">
-        <v>3.907749666197293e-05</v>
+        <v>0.0001478949966988745</v>
       </c>
       <c r="L16" t="n">
-        <v>0.01199546485260771</v>
+        <v>0.013</v>
       </c>
       <c r="M16" t="n">
-        <v>28.9942626953125</v>
+        <v>17.4560546875</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Anole</t>
+          <t>Tokay</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ACsb30learSOAEwfA2.mat</t>
+          <t>tokay_GG1rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2783.16650390625</v>
+        <v>1779.1748046875</v>
       </c>
       <c r="E17" t="n">
-        <v>7.268278767219267</v>
+        <v>11.52156691459972</v>
       </c>
       <c r="F17" t="n">
-        <v>0.5142485626019108</v>
+        <v>0.2092066714558844</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0026115141717242</v>
+        <v>0.006475792532720472</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0001847710375502683</v>
+        <v>0.0001175863500903331</v>
       </c>
       <c r="I17" t="n">
-        <v>1.141272907820804</v>
+        <v>0.8365661984221849</v>
       </c>
       <c r="J17" t="n">
-        <v>0.1502030086969103</v>
+        <v>0.02338953973482344</v>
       </c>
       <c r="K17" t="n">
-        <v>5.226451848124019e-05</v>
+        <v>1.559219156696564e-05</v>
       </c>
       <c r="L17" t="n">
-        <v>0.009002267573696146</v>
+        <v>0.021</v>
       </c>
       <c r="M17" t="n">
-        <v>25.0548095703125</v>
+        <v>37.3626708984375</v>
       </c>
     </row>
     <row r="18">
@@ -1230,34 +1230,34 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>1342.7734375</v>
+        <v>3649.90234375</v>
       </c>
       <c r="E18" t="n">
-        <v>6.131533960577602</v>
+        <v>18.07294187460645</v>
       </c>
       <c r="F18" t="n">
-        <v>0.4593700147730712</v>
+        <v>0.546884201768036</v>
       </c>
       <c r="G18" t="n">
-        <v>0.004566320564095612</v>
+        <v>0.004951623405912244</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0003421053782746363</v>
+        <v>0.0001498352970195235</v>
       </c>
       <c r="I18" t="n">
-        <v>0.6492183620177698</v>
+        <v>0.6863732722686667</v>
       </c>
       <c r="J18" t="n">
-        <v>0.06330381715723586</v>
+        <v>0.02592851099803632</v>
       </c>
       <c r="K18" t="n">
-        <v>0.0001478949966988745</v>
+        <v>3.491853465579406e-05</v>
       </c>
       <c r="L18" t="n">
-        <v>0.013</v>
+        <v>0.014</v>
       </c>
       <c r="M18" t="n">
-        <v>17.4560546875</v>
+        <v>51.09863281249999</v>
       </c>
     </row>
     <row r="19">
@@ -1275,34 +1275,34 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>1779.1748046875</v>
+        <v>4211.425781249999</v>
       </c>
       <c r="E19" t="n">
-        <v>11.52156691459972</v>
+        <v>42.41446700661243</v>
       </c>
       <c r="F19" t="n">
-        <v>0.2092066714558844</v>
+        <v>1.116815656601959</v>
       </c>
       <c r="G19" t="n">
-        <v>0.006475792532720472</v>
+        <v>0.0100712844555991</v>
       </c>
       <c r="H19" t="n">
-        <v>0.0001175863500903331</v>
+        <v>0.0002651870683734276</v>
       </c>
       <c r="I19" t="n">
-        <v>0.8365661984221849</v>
+        <v>0.6961851696660399</v>
       </c>
       <c r="J19" t="n">
-        <v>0.02338953973482344</v>
+        <v>0.02016588878326316</v>
       </c>
       <c r="K19" t="n">
-        <v>1.559219156696564e-05</v>
+        <v>9.081672769912088e-05</v>
       </c>
       <c r="L19" t="n">
-        <v>0.021</v>
+        <v>0.027</v>
       </c>
       <c r="M19" t="n">
-        <v>37.3626708984375</v>
+        <v>113.70849609375</v>
       </c>
     </row>
     <row r="20">
@@ -1312,42 +1312,42 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>tokay_GG1rearSOAEwf.mat</t>
+          <t>tokay_GG2rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>3649.90234375</v>
+        <v>1364.1357421875</v>
       </c>
       <c r="E20" t="n">
-        <v>18.07294187460645</v>
+        <v>6.846207063358801</v>
       </c>
       <c r="F20" t="n">
-        <v>0.546884201768036</v>
+        <v>0.4189574574885184</v>
       </c>
       <c r="G20" t="n">
-        <v>0.004951623405912244</v>
+        <v>0.005018713938526649</v>
       </c>
       <c r="H20" t="n">
-        <v>0.0001498352970195235</v>
+        <v>0.0003071229970242455</v>
       </c>
       <c r="I20" t="n">
-        <v>0.6863732722686667</v>
+        <v>0.5547149042899115</v>
       </c>
       <c r="J20" t="n">
-        <v>0.02592851099803632</v>
+        <v>0.05541872253904787</v>
       </c>
       <c r="K20" t="n">
-        <v>3.491853465579406e-05</v>
+        <v>4.802994423830783e-05</v>
       </c>
       <c r="L20" t="n">
-        <v>0.014</v>
+        <v>0.017</v>
       </c>
       <c r="M20" t="n">
-        <v>51.09863281249999</v>
+        <v>23.1903076171875</v>
       </c>
     </row>
     <row r="21">
@@ -1357,42 +1357,42 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>tokay_GG1rearSOAEwf.mat</t>
+          <t>tokay_GG2rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>4211.425781249999</v>
+        <v>1776.123046875</v>
       </c>
       <c r="E21" t="n">
-        <v>42.41446700661243</v>
+        <v>13.38916641103127</v>
       </c>
       <c r="F21" t="n">
-        <v>1.116815656601959</v>
+        <v>1.137979390761663</v>
       </c>
       <c r="G21" t="n">
-        <v>0.0100712844555991</v>
+        <v>0.007538422765578569</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0002651870683734276</v>
+        <v>0.0006407097710735084</v>
       </c>
       <c r="I21" t="n">
-        <v>0.6961851696660399</v>
+        <v>0.3591500973523799</v>
       </c>
       <c r="J21" t="n">
-        <v>0.02016588878326316</v>
+        <v>0.02591332113657915</v>
       </c>
       <c r="K21" t="n">
-        <v>9.081672769912088e-05</v>
+        <v>0.0001935010696527881</v>
       </c>
       <c r="L21" t="n">
-        <v>0.027</v>
+        <v>0.015</v>
       </c>
       <c r="M21" t="n">
-        <v>113.70849609375</v>
+        <v>26.641845703125</v>
       </c>
     </row>
     <row r="22">
@@ -1410,34 +1410,34 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>1364.1357421875</v>
+        <v>3607.177734375</v>
       </c>
       <c r="E22" t="n">
-        <v>6.846207063358801</v>
+        <v>25.36319341857883</v>
       </c>
       <c r="F22" t="n">
-        <v>0.4189574574885184</v>
+        <v>0.3885983005927728</v>
       </c>
       <c r="G22" t="n">
-        <v>0.005018713938526649</v>
+        <v>0.007031312368358639</v>
       </c>
       <c r="H22" t="n">
-        <v>0.0003071229970242455</v>
+        <v>0.0001077291803199998</v>
       </c>
       <c r="I22" t="n">
-        <v>0.5547149042899115</v>
+        <v>0.9266748780218937</v>
       </c>
       <c r="J22" t="n">
-        <v>0.05541872253904787</v>
+        <v>0.016927262403673</v>
       </c>
       <c r="K22" t="n">
-        <v>4.802994423830783e-05</v>
+        <v>3.064960074417074e-05</v>
       </c>
       <c r="L22" t="n">
-        <v>0.017</v>
+        <v>0.02</v>
       </c>
       <c r="M22" t="n">
-        <v>23.1903076171875</v>
+        <v>72.14355468749999</v>
       </c>
     </row>
     <row r="23">
@@ -1455,34 +1455,34 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1776.123046875</v>
+        <v>4394.531249999999</v>
       </c>
       <c r="E23" t="n">
-        <v>13.38916641103127</v>
+        <v>18.78603307275305</v>
       </c>
       <c r="F23" t="n">
-        <v>1.137979390761663</v>
+        <v>1.099972437977817</v>
       </c>
       <c r="G23" t="n">
-        <v>0.007538422765578569</v>
+        <v>0.004274866192555362</v>
       </c>
       <c r="H23" t="n">
-        <v>0.0006407097710735084</v>
+        <v>0.000250304839219841</v>
       </c>
       <c r="I23" t="n">
-        <v>0.3591500973523799</v>
+        <v>0.8803627845908035</v>
       </c>
       <c r="J23" t="n">
-        <v>0.02591332113657915</v>
+        <v>0.08180927068553458</v>
       </c>
       <c r="K23" t="n">
-        <v>0.0001935010696527881</v>
+        <v>9.33585981801773e-05</v>
       </c>
       <c r="L23" t="n">
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="M23" t="n">
-        <v>26.641845703125</v>
+        <v>61.52343749999999</v>
       </c>
     </row>
     <row r="24">
@@ -1492,42 +1492,42 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>tokay_GG2rearSOAEwf.mat</t>
+          <t>tokay_GG3rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>3607.177734375</v>
+        <v>1257.32421875</v>
       </c>
       <c r="E24" t="n">
-        <v>25.36319341857883</v>
+        <v>11.62346449124788</v>
       </c>
       <c r="F24" t="n">
-        <v>0.3885983005927728</v>
+        <v>0.1253765031284501</v>
       </c>
       <c r="G24" t="n">
-        <v>0.007031312368358639</v>
+        <v>0.009244603991485696</v>
       </c>
       <c r="H24" t="n">
-        <v>0.0001077291803199998</v>
+        <v>9.971692365322947e-05</v>
       </c>
       <c r="I24" t="n">
-        <v>0.9266748780218937</v>
+        <v>0.5513895841222959</v>
       </c>
       <c r="J24" t="n">
-        <v>0.016927262403673</v>
+        <v>0.006931187990993423</v>
       </c>
       <c r="K24" t="n">
-        <v>3.064960074417074e-05</v>
+        <v>8.934594135322911e-06</v>
       </c>
       <c r="L24" t="n">
-        <v>0.02</v>
+        <v>0.028</v>
       </c>
       <c r="M24" t="n">
-        <v>72.14355468749999</v>
+        <v>35.20507812499999</v>
       </c>
     </row>
     <row r="25">
@@ -1537,42 +1537,42 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>tokay_GG2rearSOAEwf.mat</t>
+          <t>tokay_GG3rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>4394.531249999999</v>
+        <v>2578.7353515625</v>
       </c>
       <c r="E25" t="n">
-        <v>18.78603307275305</v>
+        <v>10.12264755651465</v>
       </c>
       <c r="F25" t="n">
-        <v>1.099972437977817</v>
+        <v>0.4993633105985658</v>
       </c>
       <c r="G25" t="n">
-        <v>0.004274866192555362</v>
+        <v>0.00392543094830618</v>
       </c>
       <c r="H25" t="n">
-        <v>0.000250304839219841</v>
+        <v>0.0001936465912626486</v>
       </c>
       <c r="I25" t="n">
-        <v>0.8803627845908035</v>
+        <v>0.5526520268452401</v>
       </c>
       <c r="J25" t="n">
-        <v>0.08180927068553458</v>
+        <v>0.03976386604077077</v>
       </c>
       <c r="K25" t="n">
-        <v>9.33585981801773e-05</v>
+        <v>3.942567143227363e-05</v>
       </c>
       <c r="L25" t="n">
         <v>0.014</v>
       </c>
       <c r="M25" t="n">
-        <v>61.52343749999999</v>
+        <v>36.10229492187499</v>
       </c>
     </row>
     <row r="26">
@@ -1590,34 +1590,34 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>1257.32421875</v>
+        <v>3567.5048828125</v>
       </c>
       <c r="E26" t="n">
-        <v>11.62346449124788</v>
+        <v>22.51277151151663</v>
       </c>
       <c r="F26" t="n">
-        <v>0.1253765031284501</v>
+        <v>0.4729479126697034</v>
       </c>
       <c r="G26" t="n">
-        <v>0.009244603991485696</v>
+        <v>0.006310508955426664</v>
       </c>
       <c r="H26" t="n">
-        <v>9.971692365322947e-05</v>
+        <v>0.0001325710624667309</v>
       </c>
       <c r="I26" t="n">
-        <v>0.5513895841222959</v>
+        <v>0.864825305499054</v>
       </c>
       <c r="J26" t="n">
-        <v>0.006931187990993423</v>
+        <v>0.02281395465232204</v>
       </c>
       <c r="K26" t="n">
-        <v>8.934594135322911e-06</v>
+        <v>3.66446269727613e-05</v>
       </c>
       <c r="L26" t="n">
-        <v>0.028</v>
+        <v>0.018</v>
       </c>
       <c r="M26" t="n">
-        <v>35.20507812499999</v>
+        <v>64.21508789062499</v>
       </c>
     </row>
     <row r="27">
@@ -1627,42 +1627,42 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>tokay_GG3rearSOAEwf.mat</t>
+          <t>tokay_GG4rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>1837.158203125</v>
+        <v>1251.220703125</v>
       </c>
       <c r="E27" t="n">
-        <v>9.933323480671556</v>
+        <v>11.33802628926189</v>
       </c>
       <c r="F27" t="n">
-        <v>0.9125675545449414</v>
+        <v>0.1925690579996052</v>
       </c>
       <c r="G27" t="n">
-        <v>0.005406896076655242</v>
+        <v>0.009061571840159361</v>
       </c>
       <c r="H27" t="n">
-        <v>0.000496727801118416</v>
+        <v>0.0001539049485983187</v>
       </c>
       <c r="I27" t="n">
-        <v>0.3588351446793495</v>
+        <v>0.6415738889345853</v>
       </c>
       <c r="J27" t="n">
-        <v>0.03232693655295812</v>
+        <v>0.01261480696215831</v>
       </c>
       <c r="K27" t="n">
-        <v>0.0001219883882150051</v>
+        <v>2.537789946157043e-05</v>
       </c>
       <c r="L27" t="n">
-        <v>0.012</v>
+        <v>0.025</v>
       </c>
       <c r="M27" t="n">
-        <v>22.0458984375</v>
+        <v>31.280517578125</v>
       </c>
     </row>
     <row r="28">
@@ -1672,42 +1672,42 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>tokay_GG3rearSOAEwf.mat</t>
+          <t>tokay_GG4rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>2578.7353515625</v>
+        <v>2590.9423828125</v>
       </c>
       <c r="E28" t="n">
-        <v>10.12264755651465</v>
+        <v>14.05842710224199</v>
       </c>
       <c r="F28" t="n">
-        <v>0.4993633105985658</v>
+        <v>0.4180973196382368</v>
       </c>
       <c r="G28" t="n">
-        <v>0.00392543094830618</v>
+        <v>0.005425989862029039</v>
       </c>
       <c r="H28" t="n">
-        <v>0.0001936465912626486</v>
+        <v>0.0001613688217892314</v>
       </c>
       <c r="I28" t="n">
-        <v>0.5526520268452401</v>
+        <v>0.9037684708219275</v>
       </c>
       <c r="J28" t="n">
-        <v>0.03976386604077077</v>
+        <v>0.04225699540827385</v>
       </c>
       <c r="K28" t="n">
-        <v>3.942567143227363e-05</v>
+        <v>4.56128719840505e-05</v>
       </c>
       <c r="L28" t="n">
-        <v>0.014</v>
+        <v>0.02</v>
       </c>
       <c r="M28" t="n">
-        <v>36.10229492187499</v>
+        <v>51.81884765624999</v>
       </c>
     </row>
     <row r="29">
@@ -1717,42 +1717,42 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>tokay_GG3rearSOAEwf.mat</t>
+          <t>tokay_GG4rearSOAEwf.mat</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3567.5048828125</v>
+        <v>3216.552734375</v>
       </c>
       <c r="E29" t="n">
-        <v>22.51277151151663</v>
+        <v>16.40876444930781</v>
       </c>
       <c r="F29" t="n">
-        <v>0.4729479126697034</v>
+        <v>0.4647135819602022</v>
       </c>
       <c r="G29" t="n">
-        <v>0.006310508955426664</v>
+        <v>0.005101350981735469</v>
       </c>
       <c r="H29" t="n">
-        <v>0.0001325710624667309</v>
+        <v>0.0001444756608507771</v>
       </c>
       <c r="I29" t="n">
-        <v>0.864825305499054</v>
+        <v>0.5131634816295925</v>
       </c>
       <c r="J29" t="n">
-        <v>0.02281395465232204</v>
+        <v>0.01801103458255992</v>
       </c>
       <c r="K29" t="n">
-        <v>3.66446269727613e-05</v>
+        <v>2.003039980570149e-05</v>
       </c>
       <c r="L29" t="n">
-        <v>0.018</v>
+        <v>0.015</v>
       </c>
       <c r="M29" t="n">
-        <v>64.21508789062499</v>
+        <v>48.24829101562499</v>
       </c>
     </row>
     <row r="30">
@@ -1770,169 +1770,169 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1251.220703125</v>
+        <v>3582.763671875</v>
       </c>
       <c r="E30" t="n">
-        <v>11.33802628926189</v>
+        <v>18.42227662818847</v>
       </c>
       <c r="F30" t="n">
-        <v>0.1925690579996052</v>
+        <v>0.449508661349322</v>
       </c>
       <c r="G30" t="n">
-        <v>0.009061571840159361</v>
+        <v>0.005141917892269847</v>
       </c>
       <c r="H30" t="n">
-        <v>0.0001539049485983187</v>
+        <v>0.0001254642232972282</v>
       </c>
       <c r="I30" t="n">
-        <v>0.6415738889345853</v>
+        <v>0.8683443504099395</v>
       </c>
       <c r="J30" t="n">
-        <v>0.01261480696215831</v>
+        <v>0.0261224419154641</v>
       </c>
       <c r="K30" t="n">
-        <v>2.537789946157043e-05</v>
+        <v>4.308109283493859e-05</v>
       </c>
       <c r="L30" t="n">
-        <v>0.025</v>
+        <v>0.015</v>
       </c>
       <c r="M30" t="n">
-        <v>31.280517578125</v>
+        <v>53.74145507812499</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Tokay</t>
+          <t>Owl</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>tokay_GG4rearSOAEwf.mat</t>
+          <t>Owl2R1.mat</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>2590.9423828125</v>
+        <v>4350.5859375</v>
       </c>
       <c r="E31" t="n">
-        <v>14.05842710224199</v>
+        <v>15.9047916367591</v>
       </c>
       <c r="F31" t="n">
-        <v>0.4180973196382368</v>
+        <v>1.423485180873561</v>
       </c>
       <c r="G31" t="n">
-        <v>0.005425989862029039</v>
+        <v>0.003655781512018252</v>
       </c>
       <c r="H31" t="n">
-        <v>0.0001613688217892314</v>
+        <v>0.0003271939001603876</v>
       </c>
       <c r="I31" t="n">
-        <v>0.9037684708219275</v>
+        <v>0.5720619479951752</v>
       </c>
       <c r="J31" t="n">
-        <v>0.04225699540827385</v>
+        <v>0.0625345527309798</v>
       </c>
       <c r="K31" t="n">
-        <v>4.56128719840505e-05</v>
+        <v>0.0001353069274301281</v>
       </c>
       <c r="L31" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="M31" t="n">
-        <v>51.81884765624999</v>
+        <v>43.505859375</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Tokay</t>
+          <t>Owl</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>tokay_GG4rearSOAEwf.mat</t>
+          <t>Owl2R1.mat</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>3216.552734375</v>
+        <v>7453.125</v>
       </c>
       <c r="E32" t="n">
-        <v>16.40876444930781</v>
+        <v>27.89797667104672</v>
       </c>
       <c r="F32" t="n">
-        <v>0.4647135819602022</v>
+        <v>1.153389827536741</v>
       </c>
       <c r="G32" t="n">
-        <v>0.005101350981735469</v>
+        <v>0.003743124752509413</v>
       </c>
       <c r="H32" t="n">
-        <v>0.0001444756608507771</v>
+        <v>0.0001547525135479065</v>
       </c>
       <c r="I32" t="n">
-        <v>0.5131634816295925</v>
+        <v>0.8325065520250786</v>
       </c>
       <c r="J32" t="n">
-        <v>0.01801103458255992</v>
+        <v>0.05181307322741659</v>
       </c>
       <c r="K32" t="n">
-        <v>2.003039980570149e-05</v>
+        <v>5.636892375331214e-05</v>
       </c>
       <c r="L32" t="n">
-        <v>0.015</v>
+        <v>0.014</v>
       </c>
       <c r="M32" t="n">
-        <v>48.24829101562499</v>
+        <v>104.34375</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Tokay</t>
+          <t>Owl</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>tokay_GG4rearSOAEwf.mat</t>
+          <t>Owl2R1.mat</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3582.763671875</v>
+        <v>8452.1484375</v>
       </c>
       <c r="E33" t="n">
-        <v>18.42227662818847</v>
+        <v>28.6867161513073</v>
       </c>
       <c r="F33" t="n">
-        <v>0.449508661349322</v>
+        <v>1.876291015361221</v>
       </c>
       <c r="G33" t="n">
-        <v>0.005141917892269847</v>
+        <v>0.003394014712760101</v>
       </c>
       <c r="H33" t="n">
-        <v>0.0001254642232972282</v>
+        <v>0.0002219898324355737</v>
       </c>
       <c r="I33" t="n">
-        <v>0.8683443504099395</v>
+        <v>1.00679946801934</v>
       </c>
       <c r="J33" t="n">
-        <v>0.0261224419154641</v>
+        <v>0.08466789455859021</v>
       </c>
       <c r="K33" t="n">
-        <v>4.308109283493859e-05</v>
+        <v>0.0002007681358037239</v>
       </c>
       <c r="L33" t="n">
-        <v>0.015</v>
+        <v>0.01</v>
       </c>
       <c r="M33" t="n">
-        <v>53.74145507812499</v>
+        <v>84.521484375</v>
       </c>
     </row>
     <row r="34">
@@ -1950,34 +1950,34 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>4350.5859375</v>
+        <v>9026.3671875</v>
       </c>
       <c r="E34" t="n">
-        <v>15.9047916367591</v>
+        <v>40.82500061358546</v>
       </c>
       <c r="F34" t="n">
-        <v>1.423485180873561</v>
+        <v>1.33290471134739</v>
       </c>
       <c r="G34" t="n">
-        <v>0.003655781512018252</v>
+        <v>0.004522860611090718</v>
       </c>
       <c r="H34" t="n">
-        <v>0.0003271939001603876</v>
+        <v>0.0001476679026744268</v>
       </c>
       <c r="I34" t="n">
-        <v>0.5720619479951752</v>
+        <v>0.9365272905858708</v>
       </c>
       <c r="J34" t="n">
-        <v>0.0625345527309798</v>
+        <v>0.03425364759579562</v>
       </c>
       <c r="K34" t="n">
-        <v>0.0001353069274301281</v>
+        <v>0.0001019660249389289</v>
       </c>
       <c r="L34" t="n">
-        <v>0.01</v>
+        <v>0.013</v>
       </c>
       <c r="M34" t="n">
-        <v>43.505859375</v>
+        <v>117.3427734375</v>
       </c>
     </row>
     <row r="35">
@@ -1987,42 +1987,42 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Owl2R1.mat</t>
+          <t>Owl7L1.mat</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>7453.125</v>
+        <v>6837.890625</v>
       </c>
       <c r="E35" t="n">
-        <v>27.89797667104672</v>
+        <v>23.60324382350569</v>
       </c>
       <c r="F35" t="n">
-        <v>1.153389827536741</v>
+        <v>1.106831619203418</v>
       </c>
       <c r="G35" t="n">
-        <v>0.003743124752509413</v>
+        <v>0.003451831144711486</v>
       </c>
       <c r="H35" t="n">
-        <v>0.0001547525135479065</v>
+        <v>0.0001618674061788488</v>
       </c>
       <c r="I35" t="n">
-        <v>0.8325065520250786</v>
+        <v>0.7702004783810436</v>
       </c>
       <c r="J35" t="n">
-        <v>0.05181307322741659</v>
+        <v>0.05590319239940636</v>
       </c>
       <c r="K35" t="n">
-        <v>5.636892375331214e-05</v>
+        <v>3.473496131142383e-05</v>
       </c>
       <c r="L35" t="n">
-        <v>0.014</v>
+        <v>0.011</v>
       </c>
       <c r="M35" t="n">
-        <v>104.34375</v>
+        <v>75.216796875</v>
       </c>
     </row>
     <row r="36">
@@ -2032,42 +2032,42 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Owl2R1.mat</t>
+          <t>Owl7L1.mat</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>8452.1484375</v>
+        <v>7901.3671875</v>
       </c>
       <c r="E36" t="n">
-        <v>28.6867161513073</v>
+        <v>39.41444689003371</v>
       </c>
       <c r="F36" t="n">
-        <v>1.876291015361221</v>
+        <v>0.9452817831303912</v>
       </c>
       <c r="G36" t="n">
-        <v>0.003394014712760101</v>
+        <v>0.004988307207439689</v>
       </c>
       <c r="H36" t="n">
-        <v>0.0002219898324355737</v>
+        <v>0.0001196352176400347</v>
       </c>
       <c r="I36" t="n">
-        <v>1.00679946801934</v>
+        <v>0.7954598749435153</v>
       </c>
       <c r="J36" t="n">
-        <v>0.08466789455859021</v>
+        <v>0.02761396046219513</v>
       </c>
       <c r="K36" t="n">
-        <v>0.0002007681358037239</v>
+        <v>2.232822505732376e-05</v>
       </c>
       <c r="L36" t="n">
-        <v>0.01</v>
+        <v>0.016</v>
       </c>
       <c r="M36" t="n">
-        <v>84.521484375</v>
+        <v>126.421875</v>
       </c>
     </row>
     <row r="37">
@@ -2077,42 +2077,42 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Owl2R1.mat</t>
+          <t>Owl7L1.mat</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>9026.3671875</v>
+        <v>8835.9375</v>
       </c>
       <c r="E37" t="n">
-        <v>40.82500061358546</v>
+        <v>35.72053899303256</v>
       </c>
       <c r="F37" t="n">
-        <v>1.33290471134739</v>
+        <v>1.074154812246839</v>
       </c>
       <c r="G37" t="n">
-        <v>0.004522860611090718</v>
+        <v>0.0040426427861257</v>
       </c>
       <c r="H37" t="n">
-        <v>0.0001476679026744268</v>
+        <v>0.0001215665923674584</v>
       </c>
       <c r="I37" t="n">
-        <v>0.9365272905858708</v>
+        <v>1.04280508250793</v>
       </c>
       <c r="J37" t="n">
-        <v>0.03425364759579562</v>
+        <v>0.04443048827109366</v>
       </c>
       <c r="K37" t="n">
-        <v>0.0001019660249389289</v>
+        <v>4.975896683053984e-05</v>
       </c>
       <c r="L37" t="n">
         <v>0.013</v>
       </c>
       <c r="M37" t="n">
-        <v>117.3427734375</v>
+        <v>114.8671875</v>
       </c>
     </row>
     <row r="38">
@@ -2130,34 +2130,34 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>6837.890625</v>
+        <v>9257.8125</v>
       </c>
       <c r="E38" t="n">
-        <v>23.60324382350569</v>
+        <v>21.74130783429559</v>
       </c>
       <c r="F38" t="n">
-        <v>1.106831619203418</v>
+        <v>2.216351984478953</v>
       </c>
       <c r="G38" t="n">
-        <v>0.003451831144711486</v>
+        <v>0.0023484281880083</v>
       </c>
       <c r="H38" t="n">
-        <v>0.0001618674061788488</v>
+        <v>0.0002394034211082751</v>
       </c>
       <c r="I38" t="n">
-        <v>0.7702004783810436</v>
+        <v>0.9042090629379619</v>
       </c>
       <c r="J38" t="n">
-        <v>0.05590319239940636</v>
+        <v>0.1490603075803619</v>
       </c>
       <c r="K38" t="n">
-        <v>3.473496131142383e-05</v>
+        <v>0.0001154160433088741</v>
       </c>
       <c r="L38" t="n">
-        <v>0.011</v>
+        <v>0.008</v>
       </c>
       <c r="M38" t="n">
-        <v>75.216796875</v>
+        <v>74.0625</v>
       </c>
     </row>
     <row r="39">
@@ -2167,42 +2167,42 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Owl7L1.mat</t>
+          <t>TAG6rearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>7901.3671875</v>
+        <v>5625.54931640625</v>
       </c>
       <c r="E39" t="n">
-        <v>39.41444689003371</v>
+        <v>34.65546925180981</v>
       </c>
       <c r="F39" t="n">
-        <v>0.9452817831303912</v>
+        <v>1.032392253259833</v>
       </c>
       <c r="G39" t="n">
-        <v>0.004988307207439689</v>
+        <v>0.006160370712730439</v>
       </c>
       <c r="H39" t="n">
-        <v>0.0001196352176400347</v>
+        <v>0.0001835184788530754</v>
       </c>
       <c r="I39" t="n">
-        <v>0.7954598749435153</v>
+        <v>0.6034797319092717</v>
       </c>
       <c r="J39" t="n">
-        <v>0.02761396046219513</v>
+        <v>0.0226974244216601</v>
       </c>
       <c r="K39" t="n">
-        <v>2.232822505732376e-05</v>
+        <v>3.150602982721983e-05</v>
       </c>
       <c r="L39" t="n">
-        <v>0.016</v>
+        <v>0.01700680272108844</v>
       </c>
       <c r="M39" t="n">
-        <v>126.421875</v>
+        <v>95.67260742187501</v>
       </c>
     </row>
     <row r="40">
@@ -2212,42 +2212,42 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Owl7L1.mat</t>
+          <t>TAG6rearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>8835.9375</v>
+        <v>8096.484375</v>
       </c>
       <c r="E40" t="n">
-        <v>35.72053899303256</v>
+        <v>31.54276122708445</v>
       </c>
       <c r="F40" t="n">
-        <v>1.074154812246839</v>
+        <v>1.736068953874352</v>
       </c>
       <c r="G40" t="n">
-        <v>0.0040426427861257</v>
+        <v>0.003895858963735041</v>
       </c>
       <c r="H40" t="n">
-        <v>0.0001215665923674584</v>
+        <v>0.0002144225658280668</v>
       </c>
       <c r="I40" t="n">
-        <v>1.04280508250793</v>
+        <v>0.9078887951995183</v>
       </c>
       <c r="J40" t="n">
-        <v>0.04443048827109366</v>
+        <v>0.07168539027111559</v>
       </c>
       <c r="K40" t="n">
-        <v>4.975896683053984e-05</v>
+        <v>0.0001024463198190065</v>
       </c>
       <c r="L40" t="n">
-        <v>0.013</v>
+        <v>0.01199546485260771</v>
       </c>
       <c r="M40" t="n">
-        <v>114.8671875</v>
+        <v>97.12109375</v>
       </c>
     </row>
     <row r="41">
@@ -2257,42 +2257,42 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Owl7L1.mat</t>
+          <t>TAG6rearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>9257.8125</v>
+        <v>8489.46533203125</v>
       </c>
       <c r="E41" t="n">
-        <v>21.74130783429559</v>
+        <v>67.12832638952054</v>
       </c>
       <c r="F41" t="n">
-        <v>2.216351984478953</v>
+        <v>0.7653902219417137</v>
       </c>
       <c r="G41" t="n">
-        <v>0.0023484281880083</v>
+        <v>0.007907250193512357</v>
       </c>
       <c r="H41" t="n">
-        <v>0.0002394034211082751</v>
+        <v>9.015764739080229e-05</v>
       </c>
       <c r="I41" t="n">
-        <v>0.9042090629379619</v>
+        <v>0.9675942659614759</v>
       </c>
       <c r="J41" t="n">
-        <v>0.1490603075803619</v>
+        <v>0.01253138393993231</v>
       </c>
       <c r="K41" t="n">
-        <v>0.0001154160433088741</v>
+        <v>2.610870911953302e-05</v>
       </c>
       <c r="L41" t="n">
-        <v>0.008</v>
+        <v>0.02299319727891156</v>
       </c>
       <c r="M41" t="n">
-        <v>74.0625</v>
+        <v>195.199951171875</v>
       </c>
     </row>
     <row r="42">
@@ -2310,34 +2310,34 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>5625.54931640625</v>
+        <v>9864.898681640625</v>
       </c>
       <c r="E42" t="n">
-        <v>34.65546925180981</v>
+        <v>37.13448813534781</v>
       </c>
       <c r="F42" t="n">
-        <v>1.032392253259833</v>
+        <v>2.32274022212799</v>
       </c>
       <c r="G42" t="n">
-        <v>0.006160370712730439</v>
+        <v>0.003764305071318988</v>
       </c>
       <c r="H42" t="n">
-        <v>0.0001835184788530754</v>
+        <v>0.0002354550509931539</v>
       </c>
       <c r="I42" t="n">
-        <v>0.6034797319092717</v>
+        <v>0.9020370318017126</v>
       </c>
       <c r="J42" t="n">
-        <v>0.0226974244216601</v>
+        <v>0.08170691470702759</v>
       </c>
       <c r="K42" t="n">
-        <v>3.150602982721983e-05</v>
+        <v>0.0001011302892465221</v>
       </c>
       <c r="L42" t="n">
-        <v>0.01700680272108844</v>
+        <v>0.01099773242630385</v>
       </c>
       <c r="M42" t="n">
-        <v>95.67260742187501</v>
+        <v>108.4915161132812</v>
       </c>
     </row>
     <row r="43">
@@ -2347,42 +2347,42 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>TAG6rearSOAEwf1.mat</t>
+          <t>owl_TAG4learSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>8096.484375</v>
+        <v>4944.561767578125</v>
       </c>
       <c r="E43" t="n">
-        <v>31.54276122708445</v>
+        <v>18.29297541655268</v>
       </c>
       <c r="F43" t="n">
-        <v>1.736068953874352</v>
+        <v>0.8033393902077073</v>
       </c>
       <c r="G43" t="n">
-        <v>0.003895858963735041</v>
+        <v>0.00369961510775356</v>
       </c>
       <c r="H43" t="n">
-        <v>0.0002144225658280668</v>
+        <v>0.000162469279982559</v>
       </c>
       <c r="I43" t="n">
-        <v>0.9078887951995183</v>
+        <v>0.7870901896256317</v>
       </c>
       <c r="J43" t="n">
-        <v>0.07168539027111559</v>
+        <v>0.05146404818915367</v>
       </c>
       <c r="K43" t="n">
-        <v>0.0001024463198190065</v>
+        <v>4.427669350290799e-05</v>
       </c>
       <c r="L43" t="n">
         <v>0.01199546485260771</v>
       </c>
       <c r="M43" t="n">
-        <v>97.12109375</v>
+        <v>59.31231689453125</v>
       </c>
     </row>
     <row r="44">
@@ -2392,42 +2392,42 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TAG6rearSOAEwf1.mat</t>
+          <t>owl_TAG4learSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>8489.46533203125</v>
+        <v>5768.206787109375</v>
       </c>
       <c r="E44" t="n">
-        <v>67.12832638952054</v>
+        <v>51.611743965363</v>
       </c>
       <c r="F44" t="n">
-        <v>0.7653902219417137</v>
+        <v>0.8609974135084604</v>
       </c>
       <c r="G44" t="n">
-        <v>0.007907250193512357</v>
+        <v>0.008947623736497011</v>
       </c>
       <c r="H44" t="n">
-        <v>9.015764739080229e-05</v>
+        <v>0.0001492660449401004</v>
       </c>
       <c r="I44" t="n">
-        <v>0.9675942659614759</v>
+        <v>0.7335433805796451</v>
       </c>
       <c r="J44" t="n">
-        <v>0.01253138393993231</v>
+        <v>0.01290225928639373</v>
       </c>
       <c r="K44" t="n">
-        <v>2.610870911953302e-05</v>
+        <v>3.713946382836078e-05</v>
       </c>
       <c r="L44" t="n">
         <v>0.02299319727891156</v>
       </c>
       <c r="M44" t="n">
-        <v>195.199951171875</v>
+        <v>132.6295166015625</v>
       </c>
     </row>
     <row r="45">
@@ -2437,42 +2437,42 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TAG6rearSOAEwf1.mat</t>
+          <t>owl_TAG4learSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>9864.898681640625</v>
+        <v>7184.014892578125</v>
       </c>
       <c r="E45" t="n">
-        <v>37.13448813534781</v>
+        <v>215.6276370067336</v>
       </c>
       <c r="F45" t="n">
-        <v>2.32274022212799</v>
+        <v>3.034712671861394</v>
       </c>
       <c r="G45" t="n">
-        <v>0.003764305071318988</v>
+        <v>0.03001492065801542</v>
       </c>
       <c r="H45" t="n">
-        <v>0.0002354550509931539</v>
+        <v>0.000422425721165554</v>
       </c>
       <c r="I45" t="n">
-        <v>0.9020370318017126</v>
+        <v>1.130366381225919</v>
       </c>
       <c r="J45" t="n">
-        <v>0.08170691470702759</v>
+        <v>0.01400792500779606</v>
       </c>
       <c r="K45" t="n">
-        <v>0.0001011302892465221</v>
+        <v>0.0003266917960154298</v>
       </c>
       <c r="L45" t="n">
-        <v>0.01099773242630385</v>
+        <v>0.06900226757369614</v>
       </c>
       <c r="M45" t="n">
-        <v>108.4915161132812</v>
+        <v>495.7133178710937</v>
       </c>
     </row>
     <row r="46">
@@ -2490,169 +2490,169 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4944.561767578125</v>
+        <v>9633.416748046875</v>
       </c>
       <c r="E46" t="n">
-        <v>18.29297541655268</v>
+        <v>135.9593632964347</v>
       </c>
       <c r="F46" t="n">
-        <v>0.8033393902077073</v>
+        <v>0.4672219016222747</v>
       </c>
       <c r="G46" t="n">
-        <v>0.00369961510775356</v>
+        <v>0.01411330650924032</v>
       </c>
       <c r="H46" t="n">
-        <v>0.000162469279982559</v>
+        <v>4.850012346003836e-05</v>
       </c>
       <c r="I46" t="n">
-        <v>0.7870901896256317</v>
+        <v>1.029878129593466</v>
       </c>
       <c r="J46" t="n">
-        <v>0.05146404818915367</v>
+        <v>0.003419759382196251</v>
       </c>
       <c r="K46" t="n">
-        <v>4.427669350290799e-05</v>
+        <v>7.045406667867901e-06</v>
       </c>
       <c r="L46" t="n">
-        <v>0.01199546485260771</v>
+        <v>0.03700680272108844</v>
       </c>
       <c r="M46" t="n">
-        <v>59.31231689453125</v>
+        <v>356.501953125</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Owl</t>
+          <t>Human</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>owl_TAG4learSOAEwf1.mat</t>
+          <t>ALrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>5768.206787109375</v>
+        <v>2804.69970703125</v>
       </c>
       <c r="E47" t="n">
-        <v>51.611743965363</v>
+        <v>167.6977518928591</v>
       </c>
       <c r="F47" t="n">
-        <v>0.8609974135084604</v>
+        <v>3.882225565425057</v>
       </c>
       <c r="G47" t="n">
-        <v>0.008947623736497011</v>
+        <v>0.05979169587120102</v>
       </c>
       <c r="H47" t="n">
-        <v>0.0001492660449401004</v>
+        <v>0.00138418582056842</v>
       </c>
       <c r="I47" t="n">
-        <v>0.7335433805796451</v>
+        <v>0.2857706422108235</v>
       </c>
       <c r="J47" t="n">
-        <v>0.01290225928639373</v>
+        <v>0.008790680253189602</v>
       </c>
       <c r="K47" t="n">
-        <v>3.713946382836078e-05</v>
+        <v>4.040584176469372e-05</v>
       </c>
       <c r="L47" t="n">
-        <v>0.02299319727891156</v>
+        <v>0.1609977324263039</v>
       </c>
       <c r="M47" t="n">
-        <v>132.6295166015625</v>
+        <v>451.55029296875</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Owl</t>
+          <t>Human</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>owl_TAG4learSOAEwf1.mat</t>
+          <t>ALrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>7184.014892578125</v>
+        <v>2941.973876953125</v>
       </c>
       <c r="E48" t="n">
-        <v>215.6276370067336</v>
+        <v>222.690439352903</v>
       </c>
       <c r="F48" t="n">
-        <v>3.034712671861394</v>
+        <v>1.85893806209735</v>
       </c>
       <c r="G48" t="n">
-        <v>0.03001492065801542</v>
+        <v>0.07569422730005131</v>
       </c>
       <c r="H48" t="n">
-        <v>0.000422425721165554</v>
+        <v>0.0006318676303212357</v>
       </c>
       <c r="I48" t="n">
-        <v>1.130366381225919</v>
+        <v>0.4857636368433578</v>
       </c>
       <c r="J48" t="n">
-        <v>0.01400792500779606</v>
+        <v>0.00384554313009231</v>
       </c>
       <c r="K48" t="n">
-        <v>0.0003266917960154298</v>
+        <v>5.245232465679472e-05</v>
       </c>
       <c r="L48" t="n">
-        <v>0.06900226757369614</v>
+        <v>0.19</v>
       </c>
       <c r="M48" t="n">
-        <v>495.7133178710937</v>
+        <v>558.9750366210938</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Owl</t>
+          <t>Human</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>owl_TAG4learSOAEwf1.mat</t>
+          <t>ALrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>9633.416748046875</v>
+        <v>3862.518310546875</v>
       </c>
       <c r="E49" t="n">
-        <v>135.9593632964347</v>
+        <v>376.1429988349735</v>
       </c>
       <c r="F49" t="n">
-        <v>0.4672219016222747</v>
+        <v>1.86195496166382</v>
       </c>
       <c r="G49" t="n">
-        <v>0.01411330650924032</v>
+        <v>0.09738283901668215</v>
       </c>
       <c r="H49" t="n">
-        <v>4.850012346003836e-05</v>
+        <v>0.0004820572517623082</v>
       </c>
       <c r="I49" t="n">
-        <v>1.029878129593466</v>
+        <v>0.5013992960040554</v>
       </c>
       <c r="J49" t="n">
-        <v>0.003419759382196251</v>
+        <v>0.002032020225741199</v>
       </c>
       <c r="K49" t="n">
-        <v>7.045406667867901e-06</v>
+        <v>3.807923471616782e-05</v>
       </c>
       <c r="L49" t="n">
-        <v>0.03700680272108844</v>
+        <v>0.2470068027210884</v>
       </c>
       <c r="M49" t="n">
-        <v>356.501953125</v>
+        <v>954.0682983398438</v>
       </c>
     </row>
     <row r="50">
@@ -2662,42 +2662,42 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>ALrearSOAEwf1.mat</t>
+          <t>JIrearSOAEwf2.mat</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>2662.042236328125</v>
+        <v>2339.044189453125</v>
       </c>
       <c r="E50" t="n">
-        <v>757.6780351939651</v>
+        <v>816.2187081524804</v>
       </c>
       <c r="F50" t="n">
-        <v>516.3996991160316</v>
+        <v>2.999526586542089</v>
       </c>
       <c r="G50" t="n">
-        <v>0.284622845142782</v>
+        <v>0.3489539495802833</v>
       </c>
       <c r="H50" t="n">
-        <v>0.1939862907015048</v>
+        <v>0.001282372774343945</v>
       </c>
       <c r="I50" t="n">
-        <v>0.01868869783957859</v>
+        <v>1.082705109603358</v>
       </c>
       <c r="J50" t="n">
-        <v>0.003157301718808318</v>
+        <v>0.0031908679437738</v>
       </c>
       <c r="K50" t="n">
-        <v>2.829513251633526e-05</v>
+        <v>0.0003130492210637514</v>
       </c>
       <c r="L50" t="n">
-        <v>0.1039909297052154</v>
+        <v>0.7919954648526077</v>
       </c>
       <c r="M50" t="n">
-        <v>276.8282470703125</v>
+        <v>1852.512390136719</v>
       </c>
     </row>
     <row r="51">
@@ -2707,42 +2707,42 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>ALrearSOAEwf1.mat</t>
+          <t>JIrearSOAEwf2.mat</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>2804.69970703125</v>
+        <v>4050.933837890625</v>
       </c>
       <c r="E51" t="n">
-        <v>167.6977518928591</v>
+        <v>875.387415059495</v>
       </c>
       <c r="F51" t="n">
-        <v>3.882225565425057</v>
+        <v>2.9142914253922</v>
       </c>
       <c r="G51" t="n">
-        <v>0.05979169587120102</v>
+        <v>0.2160952141137217</v>
       </c>
       <c r="H51" t="n">
-        <v>0.00138418582056842</v>
+        <v>0.0007194122496233388</v>
       </c>
       <c r="I51" t="n">
-        <v>0.2857706422108235</v>
+        <v>0.6258624934294579</v>
       </c>
       <c r="J51" t="n">
-        <v>0.008790680253189602</v>
+        <v>0.001832888595897413</v>
       </c>
       <c r="K51" t="n">
-        <v>4.040584176469372e-05</v>
+        <v>4.807626702127727e-05</v>
       </c>
       <c r="L51" t="n">
-        <v>0.1609977324263039</v>
+        <v>0.5350113378684808</v>
       </c>
       <c r="M51" t="n">
-        <v>451.55029296875</v>
+        <v>2167.295532226562</v>
       </c>
     </row>
     <row r="52">
@@ -2752,42 +2752,42 @@
         </is>
       </c>
       <c r="B52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>ALrearSOAEwf1.mat</t>
+          <t>JIrearSOAEwf2.mat</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2941.973876953125</v>
+        <v>5838.189697265625</v>
       </c>
       <c r="E52" t="n">
-        <v>222.690439352903</v>
+        <v>570.729488728586</v>
       </c>
       <c r="F52" t="n">
-        <v>1.85893806209735</v>
+        <v>4.902349265027959</v>
       </c>
       <c r="G52" t="n">
-        <v>0.07569422730005131</v>
+        <v>0.097757955517597</v>
       </c>
       <c r="H52" t="n">
-        <v>0.0006318676303212357</v>
+        <v>0.0008397036614490316</v>
       </c>
       <c r="I52" t="n">
-        <v>0.4857636368433578</v>
+        <v>0.4885420295906551</v>
       </c>
       <c r="J52" t="n">
-        <v>0.00384554313009231</v>
+        <v>0.004515183140930636</v>
       </c>
       <c r="K52" t="n">
-        <v>5.245232465679472e-05</v>
+        <v>4.768790098019363e-05</v>
       </c>
       <c r="L52" t="n">
-        <v>0.19</v>
+        <v>0.2409977324263038</v>
       </c>
       <c r="M52" t="n">
-        <v>558.9750366210938</v>
+        <v>1406.990478515625</v>
       </c>
     </row>
     <row r="53">
@@ -2797,42 +2797,42 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ALrearSOAEwf1.mat</t>
+          <t>JIrearSOAEwf2.mat</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>3862.518310546875</v>
+        <v>8309.124755859375</v>
       </c>
       <c r="E53" t="n">
-        <v>376.1429988349735</v>
+        <v>1474.04758301067</v>
       </c>
       <c r="F53" t="n">
-        <v>1.86195496166382</v>
+        <v>6.844123938268901</v>
       </c>
       <c r="G53" t="n">
-        <v>0.09738283901668215</v>
+        <v>0.1774010652531376</v>
       </c>
       <c r="H53" t="n">
-        <v>0.0004820572517623082</v>
+        <v>0.0008236877095198992</v>
       </c>
       <c r="I53" t="n">
-        <v>0.5013992960040554</v>
+        <v>0.9855267647169658</v>
       </c>
       <c r="J53" t="n">
-        <v>0.002032020225741199</v>
+        <v>0.003543890479037869</v>
       </c>
       <c r="K53" t="n">
-        <v>3.807923471616782e-05</v>
+        <v>0.000275935823184071</v>
       </c>
       <c r="L53" t="n">
-        <v>0.2470068027210884</v>
+        <v>0.4560090702947846</v>
       </c>
       <c r="M53" t="n">
-        <v>954.0682983398438</v>
+        <v>3789.036254882812</v>
       </c>
     </row>
     <row r="54">
@@ -2842,42 +2842,42 @@
         </is>
       </c>
       <c r="B54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>JIrearSOAEwf2.mat</t>
+          <t>LSrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>2339.044189453125</v>
+        <v>732.12890625</v>
       </c>
       <c r="E54" t="n">
-        <v>816.2187081524804</v>
+        <v>480.7559039624068</v>
       </c>
       <c r="F54" t="n">
-        <v>2.999526586542089</v>
+        <v>2.590558241270873</v>
       </c>
       <c r="G54" t="n">
-        <v>0.3489539495802833</v>
+        <v>0.6566547227657791</v>
       </c>
       <c r="H54" t="n">
-        <v>0.001282372774343945</v>
+        <v>0.003538390875098538</v>
       </c>
       <c r="I54" t="n">
-        <v>1.082705109603358</v>
+        <v>0.2313446435168593</v>
       </c>
       <c r="J54" t="n">
-        <v>0.0031908679437738</v>
+        <v>0.0007995027088395416</v>
       </c>
       <c r="K54" t="n">
-        <v>0.0003130492210637514</v>
+        <v>6.505102567272299e-05</v>
       </c>
       <c r="L54" t="n">
-        <v>0.7919954648526077</v>
+        <v>1.184988662131519</v>
       </c>
       <c r="M54" t="n">
-        <v>1852.512390136719</v>
+        <v>867.564453125</v>
       </c>
     </row>
     <row r="55">
@@ -2887,42 +2887,42 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>JIrearSOAEwf2.mat</t>
+          <t>LSrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>4050.933837890625</v>
+        <v>985.14404296875</v>
       </c>
       <c r="E55" t="n">
-        <v>875.387415059495</v>
+        <v>755.1092983322764</v>
       </c>
       <c r="F55" t="n">
-        <v>2.9142914253922</v>
+        <v>5.78636679483213</v>
       </c>
       <c r="G55" t="n">
-        <v>0.2160952141137217</v>
+        <v>0.7664963349488877</v>
       </c>
       <c r="H55" t="n">
-        <v>0.0007194122496233388</v>
+        <v>0.005873625117190787</v>
       </c>
       <c r="I55" t="n">
-        <v>0.6258624934294579</v>
+        <v>0.2014650876575078</v>
       </c>
       <c r="J55" t="n">
-        <v>0.001832888595897413</v>
+        <v>0.0009437093756378963</v>
       </c>
       <c r="K55" t="n">
-        <v>4.807626702127727e-05</v>
+        <v>8.685387154243382e-05</v>
       </c>
       <c r="L55" t="n">
-        <v>0.5350113378684808</v>
+        <v>1.178004535147392</v>
       </c>
       <c r="M55" t="n">
-        <v>2167.295532226562</v>
+        <v>1160.504150390625</v>
       </c>
     </row>
     <row r="56">
@@ -2932,42 +2932,42 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>JIrearSOAEwf2.mat</t>
+          <t>LSrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>5838.189697265625</v>
+        <v>1633.831787109375</v>
       </c>
       <c r="E56" t="n">
-        <v>570.729488728586</v>
+        <v>132.9909462675353</v>
       </c>
       <c r="F56" t="n">
-        <v>4.902349265027959</v>
+        <v>3.89230636927897</v>
       </c>
       <c r="G56" t="n">
-        <v>0.097757955517597</v>
+        <v>0.08139818757157795</v>
       </c>
       <c r="H56" t="n">
-        <v>0.0008397036614490316</v>
+        <v>0.002382317690222784</v>
       </c>
       <c r="I56" t="n">
-        <v>0.4885420295906551</v>
+        <v>0.1611276796094402</v>
       </c>
       <c r="J56" t="n">
-        <v>0.004515183140930636</v>
+        <v>0.004508124343530481</v>
       </c>
       <c r="K56" t="n">
-        <v>4.768790098019363e-05</v>
+        <v>3.981241815961933e-05</v>
       </c>
       <c r="L56" t="n">
-        <v>0.2409977324263038</v>
+        <v>0.1580045351473923</v>
       </c>
       <c r="M56" t="n">
-        <v>1406.990478515625</v>
+        <v>258.15283203125</v>
       </c>
     </row>
     <row r="57">
@@ -2977,42 +2977,42 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>JIrearSOAEwf2.mat</t>
+          <t>LSrearSOAEwf1.mat</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>8309.124755859375</v>
+        <v>2225.994873046875</v>
       </c>
       <c r="E57" t="n">
-        <v>1474.04758301067</v>
+        <v>626.8054666130253</v>
       </c>
       <c r="F57" t="n">
-        <v>6.844123938268901</v>
+        <v>3.220620718286531</v>
       </c>
       <c r="G57" t="n">
-        <v>0.1774010652531376</v>
+        <v>0.2815844161200033</v>
       </c>
       <c r="H57" t="n">
-        <v>0.0008236877095198992</v>
+        <v>0.001446823062030795</v>
       </c>
       <c r="I57" t="n">
-        <v>0.9855267647169658</v>
+        <v>0.4614251582764692</v>
       </c>
       <c r="J57" t="n">
-        <v>0.003543890479037869</v>
+        <v>0.001966584968221839</v>
       </c>
       <c r="K57" t="n">
-        <v>0.000275935823184071</v>
+        <v>8.305902471657155e-05</v>
       </c>
       <c r="L57" t="n">
-        <v>0.4560090702947846</v>
+        <v>0.6439909297052154</v>
       </c>
       <c r="M57" t="n">
-        <v>3789.036254882812</v>
+        <v>1433.5205078125</v>
       </c>
     </row>
     <row r="58">
@@ -3022,42 +3022,42 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>LSrearSOAEwf1.mat</t>
+          <t>TH13RearwaveformSOAE.mat</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>732.12890625</v>
+        <v>904.39453125</v>
       </c>
       <c r="E58" t="n">
-        <v>480.7559039624068</v>
+        <v>371.0586431441757</v>
       </c>
       <c r="F58" t="n">
-        <v>2.590558241270873</v>
+        <v>2.499614844921145</v>
       </c>
       <c r="G58" t="n">
-        <v>0.6566547227657791</v>
+        <v>0.4102840412262563</v>
       </c>
       <c r="H58" t="n">
-        <v>0.003538390875098538</v>
+        <v>0.002763854444659597</v>
       </c>
       <c r="I58" t="n">
-        <v>0.2313446435168593</v>
+        <v>0.2534923552462224</v>
       </c>
       <c r="J58" t="n">
-        <v>0.0007995027088395416</v>
+        <v>0.001104744702066296</v>
       </c>
       <c r="K58" t="n">
-        <v>6.505102567272299e-05</v>
+        <v>6.421246118393566e-05</v>
       </c>
       <c r="L58" t="n">
-        <v>1.184988662131519</v>
+        <v>0.6980045351473922</v>
       </c>
       <c r="M58" t="n">
-        <v>867.564453125</v>
+        <v>631.271484375</v>
       </c>
     </row>
     <row r="59">
@@ -3067,42 +3067,42 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LSrearSOAEwf1.mat</t>
+          <t>TH13RearwaveformSOAE.mat</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>985.14404296875</v>
+        <v>1520.782470703125</v>
       </c>
       <c r="E59" t="n">
-        <v>755.1092983322764</v>
+        <v>736.9099855362433</v>
       </c>
       <c r="F59" t="n">
-        <v>5.78636679483213</v>
+        <v>1.983253861613653</v>
       </c>
       <c r="G59" t="n">
-        <v>0.7664963349488877</v>
+        <v>0.4845597577117898</v>
       </c>
       <c r="H59" t="n">
-        <v>0.005873625117190787</v>
+        <v>0.001304100947913154</v>
       </c>
       <c r="I59" t="n">
-        <v>0.2014650876575078</v>
+        <v>0.4705307305475712</v>
       </c>
       <c r="J59" t="n">
-        <v>0.0009437093756378963</v>
+        <v>0.0009026191137522416</v>
       </c>
       <c r="K59" t="n">
-        <v>8.685387154243382e-05</v>
+        <v>5.090014400846331e-05</v>
       </c>
       <c r="L59" t="n">
-        <v>1.178004535147392</v>
+        <v>1.008004535147392</v>
       </c>
       <c r="M59" t="n">
-        <v>1160.504150390625</v>
+        <v>1532.955627441406</v>
       </c>
     </row>
     <row r="60">
@@ -3112,267 +3112,42 @@
         </is>
       </c>
       <c r="B60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LSrearSOAEwf1.mat</t>
+          <t>TH13RearwaveformSOAE.mat</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1633.831787109375</v>
+        <v>2037.579345703125</v>
       </c>
       <c r="E60" t="n">
-        <v>132.9909462675353</v>
+        <v>391.4314087693493</v>
       </c>
       <c r="F60" t="n">
-        <v>3.89230636927897</v>
+        <v>1.109644736010197</v>
       </c>
       <c r="G60" t="n">
-        <v>0.08139818757157795</v>
+        <v>0.1921060937306835</v>
       </c>
       <c r="H60" t="n">
-        <v>0.002382317690222784</v>
+        <v>0.0005445897055985727</v>
       </c>
       <c r="I60" t="n">
-        <v>0.1611276796094402</v>
+        <v>0.7303823851321648</v>
       </c>
       <c r="J60" t="n">
-        <v>0.004508124343530481</v>
+        <v>0.001581809785714539</v>
       </c>
       <c r="K60" t="n">
-        <v>3.981241815961933e-05</v>
+        <v>4.99826220365896e-05</v>
       </c>
       <c r="L60" t="n">
-        <v>0.1580045351473923</v>
+        <v>0.4229931972789115</v>
       </c>
       <c r="M60" t="n">
-        <v>258.15283203125</v>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Human</t>
-        </is>
-      </c>
-      <c r="B61" t="n">
-        <v>2</v>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>LSrearSOAEwf1.mat</t>
-        </is>
-      </c>
-      <c r="D61" t="n">
-        <v>2225.994873046875</v>
-      </c>
-      <c r="E61" t="n">
-        <v>626.8054666130253</v>
-      </c>
-      <c r="F61" t="n">
-        <v>3.220620718286531</v>
-      </c>
-      <c r="G61" t="n">
-        <v>0.2815844161200033</v>
-      </c>
-      <c r="H61" t="n">
-        <v>0.001446823062030795</v>
-      </c>
-      <c r="I61" t="n">
-        <v>0.4614251582764692</v>
-      </c>
-      <c r="J61" t="n">
-        <v>0.001966584968221839</v>
-      </c>
-      <c r="K61" t="n">
-        <v>8.305902471657155e-05</v>
-      </c>
-      <c r="L61" t="n">
-        <v>0.6439909297052154</v>
-      </c>
-      <c r="M61" t="n">
-        <v>1433.5205078125</v>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Human</t>
-        </is>
-      </c>
-      <c r="B62" t="n">
-        <v>3</v>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>TH13RearwaveformSOAE.mat</t>
-        </is>
-      </c>
-      <c r="D62" t="n">
-        <v>904.39453125</v>
-      </c>
-      <c r="E62" t="n">
-        <v>371.0586431441757</v>
-      </c>
-      <c r="F62" t="n">
-        <v>2.499614844921145</v>
-      </c>
-      <c r="G62" t="n">
-        <v>0.4102840412262563</v>
-      </c>
-      <c r="H62" t="n">
-        <v>0.002763854444659597</v>
-      </c>
-      <c r="I62" t="n">
-        <v>0.2534923552462224</v>
-      </c>
-      <c r="J62" t="n">
-        <v>0.001104744702066296</v>
-      </c>
-      <c r="K62" t="n">
-        <v>6.421246118393566e-05</v>
-      </c>
-      <c r="L62" t="n">
-        <v>0.6980045351473922</v>
-      </c>
-      <c r="M62" t="n">
-        <v>631.271484375</v>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Human</t>
-        </is>
-      </c>
-      <c r="B63" t="n">
-        <v>3</v>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>TH13RearwaveformSOAE.mat</t>
-        </is>
-      </c>
-      <c r="D63" t="n">
-        <v>1520.782470703125</v>
-      </c>
-      <c r="E63" t="n">
-        <v>736.9099855362433</v>
-      </c>
-      <c r="F63" t="n">
-        <v>1.983253861613653</v>
-      </c>
-      <c r="G63" t="n">
-        <v>0.4845597577117898</v>
-      </c>
-      <c r="H63" t="n">
-        <v>0.001304100947913154</v>
-      </c>
-      <c r="I63" t="n">
-        <v>0.4705307305475712</v>
-      </c>
-      <c r="J63" t="n">
-        <v>0.0009026191137522416</v>
-      </c>
-      <c r="K63" t="n">
-        <v>5.090014400846331e-05</v>
-      </c>
-      <c r="L63" t="n">
-        <v>1.008004535147392</v>
-      </c>
-      <c r="M63" t="n">
-        <v>1532.955627441406</v>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Human</t>
-        </is>
-      </c>
-      <c r="B64" t="n">
-        <v>3</v>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>TH13RearwaveformSOAE.mat</t>
-        </is>
-      </c>
-      <c r="D64" t="n">
-        <v>2037.579345703125</v>
-      </c>
-      <c r="E64" t="n">
-        <v>391.4314087693493</v>
-      </c>
-      <c r="F64" t="n">
-        <v>1.109644736010197</v>
-      </c>
-      <c r="G64" t="n">
-        <v>0.1921060937306835</v>
-      </c>
-      <c r="H64" t="n">
-        <v>0.0005445897055985727</v>
-      </c>
-      <c r="I64" t="n">
-        <v>0.7303823851321648</v>
-      </c>
-      <c r="J64" t="n">
-        <v>0.001581809785714539</v>
-      </c>
-      <c r="K64" t="n">
-        <v>4.99826220365896e-05</v>
-      </c>
-      <c r="L64" t="n">
-        <v>0.4229931972789115</v>
-      </c>
-      <c r="M64" t="n">
         <v>861.8822021484375</v>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Human</t>
-        </is>
-      </c>
-      <c r="B65" t="n">
-        <v>3</v>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>TH13RearwaveformSOAE.mat</t>
-        </is>
-      </c>
-      <c r="D65" t="n">
-        <v>2694.342041015625</v>
-      </c>
-      <c r="E65" t="n">
-        <v>119.9564065235588</v>
-      </c>
-      <c r="F65" t="n">
-        <v>23.83243339453002</v>
-      </c>
-      <c r="G65" t="n">
-        <v>0.04452159551292215</v>
-      </c>
-      <c r="H65" t="n">
-        <v>0.008845362998361726</v>
-      </c>
-      <c r="I65" t="n">
-        <v>0.109212781965805</v>
-      </c>
-      <c r="J65" t="n">
-        <v>0.02969266345528983</v>
-      </c>
-      <c r="K65" t="n">
-        <v>5.007598654357961e-05</v>
-      </c>
-      <c r="L65" t="n">
-        <v>0.08399092970521542</v>
-      </c>
-      <c r="M65" t="n">
-        <v>226.30029296875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>